<commit_message>
docs(kitgen): link dự phòng trong hướng dẫn trỏ trang Releases
2.1.33 đã bỏ asset gộp kitgen-easy-install.zip nên dòng dự phòng cũ trỏ
thẳng vào 404. Nay trỏ trang Releases (mục Assets) — không bao giờ chết
dù tên asset còn đổi nữa.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kit-gen/teams/easy-install-guide/huong-dan-cai-dat.xlsx
+++ b/kit-gen/teams/easy-install-guide/huong-dan-cai-dat.xlsx
@@ -654,31 +654,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="001F2937"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Giải nén ra Desktop rồi mới chạy (</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="00C00000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>ĐỪNG bấm đúp trong cửa sổ xem .zip</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="001F2937"/>
-              <sz val="11"/>
-            </rPr>
-            <t>)</t>
-          </r>
+          <t>Giải nén ra Desktop rồi mới chạy (ĐỪNG bấm đúp trong cửa sổ xem .zip)</t>
         </is>
       </c>
     </row>
@@ -779,7 +755,7 @@
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Nếu link báo Not Found (bản cũ): tải bản gộp https://github.com/hihahihahoho/test-survey/releases/latest/download/kitgen-easy-install.zip</t>
+          <t>Không tải được? Mở trang Releases rồi lấy file trong mục Assets: https://github.com/hihahihahoho/test-survey/releases/latest</t>
         </is>
       </c>
       <c r="B11" s="16" t="n"/>

</xml_diff>